<commit_message>
fix: popular SKU Cliente e ID Interno en BDs de Excel y configurar fallback automatico en PDF
</commit_message>
<xml_diff>
--- a/BD_POs_Cabecera.xlsx
+++ b/BD_POs_Cabecera.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="45">
   <si>
     <t>PO</t>
   </si>
@@ -43,6 +43,9 @@
     <t>Color_Texto</t>
   </si>
   <si>
+    <t>ID_Interno</t>
+  </si>
+  <si>
     <t>26083177</t>
   </si>
   <si>
@@ -73,6 +76,9 @@
     <t>PO 2602-0711</t>
   </si>
   <si>
+    <t>URG/GALV</t>
+  </si>
+  <si>
     <t>2026-08-17</t>
   </si>
   <si>
@@ -109,13 +115,28 @@
     <t>TORONTO</t>
   </si>
   <si>
+    <t>INT-047</t>
+  </si>
+  <si>
     <t>ESTEFANIA IBARRA</t>
   </si>
   <si>
+    <t>Luis Quintana</t>
+  </si>
+  <si>
+    <t>REQ-URG</t>
+  </si>
+  <si>
     <t>ALMACEN SIGRAMA RIO XIX</t>
   </si>
   <si>
+    <t>PLANTA RIO XIX</t>
+  </si>
+  <si>
     <t>RENO 6</t>
+  </si>
+  <si>
+    <t>URGENTE GALV</t>
   </si>
   <si>
     <t>#EC2024</t>
@@ -459,10 +480,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -490,205 +511,240 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" t="s">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" t="s">
+        <v>41</v>
+      </c>
+      <c r="I3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H4" t="s">
+        <v>41</v>
+      </c>
+      <c r="I4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>41</v>
+      </c>
+      <c r="I5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D6" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+      <c r="I6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" t="s">
+        <v>34</v>
+      </c>
+      <c r="H7" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>34</v>
+      </c>
+      <c r="H8" t="s">
+        <v>41</v>
+      </c>
+      <c r="I8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
         <v>25</v>
       </c>
-      <c r="D2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H2" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="C9" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H9" t="s">
+        <v>41</v>
+      </c>
+      <c r="I9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" t="s">
         <v>26</v>
       </c>
-      <c r="D3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="C10" t="s">
         <v>27</v>
       </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D6" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I7" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" t="s">
-        <v>29</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" t="s">
-        <v>34</v>
-      </c>
-      <c r="I8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" t="s">
-        <v>34</v>
-      </c>
-      <c r="I9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" t="s">
-        <v>17</v>
-      </c>
-      <c r="B10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C10" t="s">
-        <v>25</v>
-      </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="E10">
         <v>23474</v>
       </c>
       <c r="F10" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="H10" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="I10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>39</v>
+      </c>
+      <c r="H11" t="s">
+        <v>42</v>
+      </c>
+      <c r="I11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="F12" t="s">
+        <v>38</v>
+      </c>
+      <c r="G12" t="s">
+        <v>40</v>
+      </c>
+      <c r="H12" t="s">
+        <v>41</v>
+      </c>
+      <c r="I12" t="s">
+        <v>43</v>
+      </c>
+      <c r="J12" t="s">
         <v>33</v>
-      </c>
-      <c r="H11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I11" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: actualizar descripcion/proyecto de INT-0067 a CLOUD en BD_POs_Cabecera
</commit_message>
<xml_diff>
--- a/BD_POs_Cabecera.xlsx
+++ b/BD_POs_Cabecera.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="242">
   <si>
     <t>PO</t>
   </si>
@@ -470,9 +470,6 @@
   </si>
   <si>
     <t>SWBD RENO 4</t>
-  </si>
-  <si>
-    <t>AL, SWBD CDC 736</t>
   </si>
   <si>
     <t>ESTEFANIA IBARRA</t>
@@ -1119,22 +1116,22 @@
         <v>128</v>
       </c>
       <c r="D2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F2" t="s">
+        <v>232</v>
+      </c>
+      <c r="G2" t="s">
         <v>233</v>
       </c>
-      <c r="G2" t="s">
-        <v>234</v>
-      </c>
       <c r="H2" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I2" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1148,22 +1145,22 @@
         <v>128</v>
       </c>
       <c r="D3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F3" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G3" t="s">
         <v>128</v>
       </c>
       <c r="H3" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I3" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1177,19 +1174,19 @@
         <v>129</v>
       </c>
       <c r="D4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G4" t="s">
         <v>129</v>
       </c>
       <c r="H4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1203,22 +1200,22 @@
         <v>128</v>
       </c>
       <c r="D5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G5" t="s">
         <v>128</v>
       </c>
       <c r="H5" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I5" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1232,22 +1229,22 @@
         <v>130</v>
       </c>
       <c r="D6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G6" t="s">
         <v>130</v>
       </c>
       <c r="H6" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I6" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1261,22 +1258,22 @@
         <v>128</v>
       </c>
       <c r="D7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G7" t="s">
         <v>128</v>
       </c>
       <c r="H7" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1290,22 +1287,22 @@
         <v>131</v>
       </c>
       <c r="D8" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G8" t="s">
         <v>131</v>
       </c>
       <c r="H8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1319,22 +1316,22 @@
         <v>132</v>
       </c>
       <c r="D9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F9" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G9" t="s">
         <v>132</v>
       </c>
       <c r="H9" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I9" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1348,22 +1345,22 @@
         <v>128</v>
       </c>
       <c r="D10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F10" t="s">
+        <v>232</v>
+      </c>
+      <c r="G10" t="s">
         <v>233</v>
       </c>
-      <c r="G10" t="s">
-        <v>234</v>
-      </c>
       <c r="H10" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I10" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1377,22 +1374,22 @@
         <v>130</v>
       </c>
       <c r="D11" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F11" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G11" t="s">
         <v>130</v>
       </c>
       <c r="H11" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I11" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1406,22 +1403,22 @@
         <v>130</v>
       </c>
       <c r="D12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E12" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F12" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G12" t="s">
         <v>130</v>
       </c>
       <c r="H12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1435,19 +1432,19 @@
         <v>133</v>
       </c>
       <c r="D13" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F13" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G13" t="s">
         <v>133</v>
       </c>
       <c r="H13" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I13" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1461,22 +1458,22 @@
         <v>134</v>
       </c>
       <c r="D14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E14" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F14" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G14" t="s">
         <v>134</v>
       </c>
       <c r="H14" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I14" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1490,22 +1487,22 @@
         <v>134</v>
       </c>
       <c r="D15" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F15" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G15" t="s">
         <v>134</v>
       </c>
       <c r="H15" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I15" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1519,22 +1516,22 @@
         <v>134</v>
       </c>
       <c r="D16" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E16" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F16" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G16" t="s">
         <v>134</v>
       </c>
       <c r="H16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I16" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1548,22 +1545,22 @@
         <v>130</v>
       </c>
       <c r="D17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E17" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F17" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G17" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H17" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I17" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1577,22 +1574,22 @@
         <v>130</v>
       </c>
       <c r="D18" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E18" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F18" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G18" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H18" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I18" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1606,22 +1603,22 @@
         <v>130</v>
       </c>
       <c r="D19" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G19" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I19" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1635,19 +1632,19 @@
         <v>130</v>
       </c>
       <c r="D20" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F20" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G20" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H20" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I20" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1661,22 +1658,22 @@
         <v>130</v>
       </c>
       <c r="D21" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E21" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F21" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G21" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H21" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I21" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1690,22 +1687,22 @@
         <v>130</v>
       </c>
       <c r="D22" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E22" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F22" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G22" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H22" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I22" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1719,22 +1716,22 @@
         <v>130</v>
       </c>
       <c r="D23" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E23" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F23" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G23" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H23" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I23" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1748,22 +1745,22 @@
         <v>130</v>
       </c>
       <c r="D24" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E24" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G24" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H24" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1777,22 +1774,22 @@
         <v>130</v>
       </c>
       <c r="D25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E25" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F25" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G25" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H25" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I25" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1806,22 +1803,22 @@
         <v>130</v>
       </c>
       <c r="D26" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E26" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F26" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G26" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H26" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I26" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1835,22 +1832,22 @@
         <v>130</v>
       </c>
       <c r="D27" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E27" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F27" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G27" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H27" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I27" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1864,22 +1861,22 @@
         <v>134</v>
       </c>
       <c r="D28" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E28" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F28" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G28" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H28" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I28" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1893,22 +1890,22 @@
         <v>135</v>
       </c>
       <c r="D29" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E29" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F29" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G29" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H29" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I29" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1922,22 +1919,22 @@
         <v>135</v>
       </c>
       <c r="D30" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E30" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F30" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G30" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H30" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I30" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1951,22 +1948,22 @@
         <v>135</v>
       </c>
       <c r="D31" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E31" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F31" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G31" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H31" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I31" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1980,22 +1977,22 @@
         <v>135</v>
       </c>
       <c r="D32" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E32" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F32" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G32" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H32" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I32" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -2009,22 +2006,22 @@
         <v>135</v>
       </c>
       <c r="D33" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E33" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F33" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G33" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H33" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I33" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -2038,22 +2035,22 @@
         <v>135</v>
       </c>
       <c r="D34" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E34" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F34" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G34" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H34" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I34" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -2067,22 +2064,22 @@
         <v>136</v>
       </c>
       <c r="D35" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E35" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F35" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G35" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H35" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I35" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -2096,22 +2093,22 @@
         <v>131</v>
       </c>
       <c r="D36" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F36" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G36" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H36" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I36" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -2125,22 +2122,22 @@
         <v>134</v>
       </c>
       <c r="D37" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E37" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F37" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G37" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H37" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I37" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -2154,22 +2151,22 @@
         <v>131</v>
       </c>
       <c r="D38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E38" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F38" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G38" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H38" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I38" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -2183,22 +2180,22 @@
         <v>134</v>
       </c>
       <c r="D39" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E39" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F39" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G39" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H39" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I39" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2212,22 +2209,22 @@
         <v>134</v>
       </c>
       <c r="D40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E40" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F40" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G40" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H40" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I40" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2241,22 +2238,22 @@
         <v>134</v>
       </c>
       <c r="D41" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E41" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F41" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G41" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H41" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I41" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2270,22 +2267,22 @@
         <v>134</v>
       </c>
       <c r="D42" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F42" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G42" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H42" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I42" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -2299,22 +2296,22 @@
         <v>134</v>
       </c>
       <c r="D43" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E43" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F43" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G43" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H43" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I43" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -2328,22 +2325,22 @@
         <v>137</v>
       </c>
       <c r="D44" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E44" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F44" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G44" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H44" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I44" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -2357,22 +2354,22 @@
         <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F45" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G45" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H45" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I45" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -2386,22 +2383,22 @@
         <v>131</v>
       </c>
       <c r="D46" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E46" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F46" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G46" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H46" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I46" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -2415,22 +2412,22 @@
         <v>138</v>
       </c>
       <c r="D47" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E47" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F47" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G47" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H47" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I47" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -2444,22 +2441,22 @@
         <v>138</v>
       </c>
       <c r="D48" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E48" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="F48" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G48" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H48" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="I48" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -2473,13 +2470,13 @@
         <v>136</v>
       </c>
       <c r="F49" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H49" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I49" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2493,16 +2490,16 @@
         <v>134</v>
       </c>
       <c r="F50" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G50" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H50" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I50" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2516,13 +2513,13 @@
         <v>139</v>
       </c>
       <c r="F51" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H51" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I51" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2536,16 +2533,16 @@
         <v>136</v>
       </c>
       <c r="E52" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F52" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H52" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I52" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2559,16 +2556,16 @@
         <v>139</v>
       </c>
       <c r="E53" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F53" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H53" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I53" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2582,16 +2579,16 @@
         <v>139</v>
       </c>
       <c r="F54" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G54" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H54" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I54" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2605,22 +2602,22 @@
         <v>140</v>
       </c>
       <c r="D55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E55" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="F55" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G55" t="s">
         <v>140</v>
       </c>
       <c r="H55" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I55" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2634,22 +2631,22 @@
         <v>141</v>
       </c>
       <c r="D56" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E56" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="F56" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G56" t="s">
         <v>141</v>
       </c>
       <c r="H56" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I56" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2663,22 +2660,22 @@
         <v>142</v>
       </c>
       <c r="D57" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E57" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F57" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G57" t="s">
         <v>142</v>
       </c>
       <c r="H57" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I57" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2692,22 +2689,22 @@
         <v>142</v>
       </c>
       <c r="D58" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E58" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F58" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G58" t="s">
         <v>142</v>
       </c>
       <c r="H58" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I58" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2721,22 +2718,22 @@
         <v>143</v>
       </c>
       <c r="D59" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E59" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="F59" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G59" t="s">
         <v>143</v>
       </c>
       <c r="H59" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I59" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2750,22 +2747,22 @@
         <v>144</v>
       </c>
       <c r="D60" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E60" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F60" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G60" t="s">
         <v>144</v>
       </c>
       <c r="H60" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I60" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2779,22 +2776,22 @@
         <v>144</v>
       </c>
       <c r="D61" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E61" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F61" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G61" t="s">
         <v>144</v>
       </c>
       <c r="H61" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I61" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2808,22 +2805,22 @@
         <v>145</v>
       </c>
       <c r="D62" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E62" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F62" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G62" t="s">
         <v>145</v>
       </c>
       <c r="H62" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I62" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2837,22 +2834,22 @@
         <v>131</v>
       </c>
       <c r="D63" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E63" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="F63" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G63" t="s">
         <v>131</v>
       </c>
       <c r="H63" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I63" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2866,22 +2863,22 @@
         <v>146</v>
       </c>
       <c r="D64" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E64" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="F64" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G64" t="s">
         <v>146</v>
       </c>
       <c r="H64" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I64" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2895,22 +2892,22 @@
         <v>147</v>
       </c>
       <c r="D65" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E65" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="F65" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G65" t="s">
         <v>147</v>
       </c>
       <c r="H65" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I65" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -2924,19 +2921,19 @@
         <v>144</v>
       </c>
       <c r="D66" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F66" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G66" t="s">
         <v>144</v>
       </c>
       <c r="H66" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I66" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -2950,19 +2947,19 @@
         <v>143</v>
       </c>
       <c r="D67" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F67" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G67" t="s">
         <v>143</v>
       </c>
       <c r="H67" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I67" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -2976,22 +2973,22 @@
         <v>131</v>
       </c>
       <c r="D68" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E68" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="F68" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G68" t="s">
         <v>131</v>
       </c>
       <c r="H68" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I68" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -3005,22 +3002,22 @@
         <v>141</v>
       </c>
       <c r="D69" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E69" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="F69" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G69" t="s">
         <v>141</v>
       </c>
       <c r="H69" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I69" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3034,22 +3031,22 @@
         <v>144</v>
       </c>
       <c r="D70" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E70" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F70" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G70" t="s">
         <v>144</v>
       </c>
       <c r="H70" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I70" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -3063,22 +3060,22 @@
         <v>145</v>
       </c>
       <c r="D71" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E71" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="F71" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G71" t="s">
         <v>145</v>
       </c>
       <c r="H71" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I71" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -3092,22 +3089,22 @@
         <v>131</v>
       </c>
       <c r="D72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E72" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="F72" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G72" t="s">
         <v>131</v>
       </c>
       <c r="H72" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I72" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -3121,22 +3118,22 @@
         <v>148</v>
       </c>
       <c r="D73" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E73" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="F73" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G73" t="s">
         <v>148</v>
       </c>
       <c r="H73" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I73" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -3150,22 +3147,22 @@
         <v>149</v>
       </c>
       <c r="D74" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E74" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="F74" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G74" t="s">
         <v>149</v>
       </c>
       <c r="H74" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I74" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3179,22 +3176,22 @@
         <v>150</v>
       </c>
       <c r="D75" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E75" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="F75" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G75" t="s">
         <v>150</v>
       </c>
       <c r="H75" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I75" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3208,22 +3205,22 @@
         <v>151</v>
       </c>
       <c r="D76" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E76" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F76" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G76" t="s">
         <v>151</v>
       </c>
       <c r="H76" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I76" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3237,16 +3234,16 @@
         <v>136</v>
       </c>
       <c r="E77" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="F77" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H77" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I77" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3257,25 +3254,25 @@
         <v>127</v>
       </c>
       <c r="C78" t="s">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="D78" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E78" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="F78" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G78" t="s">
-        <v>152</v>
+        <v>128</v>
       </c>
       <c r="H78" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I78" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3289,22 +3286,22 @@
         <v>131</v>
       </c>
       <c r="D79" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E79" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F79" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G79" t="s">
         <v>131</v>
       </c>
       <c r="H79" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I79" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3318,22 +3315,22 @@
         <v>135</v>
       </c>
       <c r="D80" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E80" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="F80" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G80" t="s">
         <v>135</v>
       </c>
       <c r="H80" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I80" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3347,22 +3344,22 @@
         <v>135</v>
       </c>
       <c r="D81" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E81" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F81" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G81" t="s">
         <v>135</v>
       </c>
       <c r="H81" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I81" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3376,22 +3373,22 @@
         <v>135</v>
       </c>
       <c r="D82" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="E82" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="F82" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G82" t="s">
         <v>135</v>
       </c>
       <c r="H82" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I82" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3405,22 +3402,22 @@
         <v>135</v>
       </c>
       <c r="D83" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="E83" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F83" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="G83" t="s">
         <v>135</v>
       </c>
       <c r="H83" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="I83" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: actualizar BD_Articulos con SKUs de INT-0070 y sincronizar BD_POs con INT-0070
</commit_message>
<xml_diff>
--- a/BD_POs_Cabecera.xlsx
+++ b/BD_POs_Cabecera.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="246">
   <si>
     <t>PO</t>
   </si>
@@ -289,6 +289,9 @@
     <t>26093609</t>
   </si>
   <si>
+    <t>26093636</t>
+  </si>
+  <si>
     <t>2026-08-17</t>
   </si>
   <si>
@@ -472,6 +475,9 @@
     <t>SWBD RENO 4</t>
   </si>
   <si>
+    <t>SWBDLC8</t>
+  </si>
+  <si>
     <t>ESTEFANIA IBARRA</t>
   </si>
   <si>
@@ -499,6 +505,9 @@
     <t>LORENA HERNANDEZ</t>
   </si>
   <si>
+    <t>MAURICIO DOMINGUEZ/ ESTEFANIA</t>
+  </si>
+  <si>
     <t>23199</t>
   </si>
   <si>
@@ -710,6 +719,9 @@
   </si>
   <si>
     <t>23388</t>
+  </si>
+  <si>
+    <t>23489, 23495, 23264</t>
   </si>
   <si>
     <t>ALMACEN SIGRAMA</t>
@@ -1073,7 +1085,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1110,28 +1122,28 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C2" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D2" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E2" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F2" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G2" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="H2" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I2" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1139,28 +1151,28 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H3" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I3" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1168,25 +1180,25 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D4" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="F4" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H4" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I4" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1194,28 +1206,28 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E5" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F5" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H5" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I5" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1223,28 +1235,28 @@
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E6" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F6" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H6" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I6" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1252,28 +1264,28 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D7" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E7" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F7" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H7" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I7" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1281,28 +1293,28 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E8" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F8" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H8" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I8" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1310,28 +1322,28 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D9" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E9" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F9" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H9" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I9" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1339,28 +1351,28 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D10" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E10" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F10" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G10" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="H10" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I10" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1368,28 +1380,28 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D11" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E11" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F11" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G11" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H11" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I11" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1397,28 +1409,28 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D12" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E12" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F12" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G12" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H12" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I12" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1426,25 +1438,25 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D13" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F13" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G13" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H13" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I13" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1452,28 +1464,28 @@
         <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D14" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E14" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F14" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G14" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H14" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I14" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1481,28 +1493,28 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D15" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E15" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F15" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H15" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I15" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1510,28 +1522,28 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D16" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E16" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F16" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H16" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I16" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1539,28 +1551,28 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C17" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D17" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E17" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F17" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G17" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H17" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I17" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1568,28 +1580,28 @@
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C18" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D18" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E18" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F18" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G18" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H18" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I18" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1597,28 +1609,28 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D19" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E19" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F19" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G19" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H19" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I19" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1626,25 +1638,25 @@
         <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C20" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D20" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F20" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G20" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H20" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I20" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1652,28 +1664,28 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C21" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D21" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E21" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F21" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G21" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H21" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I21" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1681,28 +1693,28 @@
         <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D22" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E22" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F22" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G22" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H22" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I22" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1710,28 +1722,28 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C23" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D23" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E23" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F23" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G23" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H23" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I23" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1739,28 +1751,28 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C24" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D24" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E24" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F24" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G24" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H24" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I24" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1768,28 +1780,28 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D25" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E25" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F25" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G25" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H25" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I25" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1797,28 +1809,28 @@
         <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D26" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E26" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F26" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G26" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H26" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I26" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1826,28 +1838,28 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C27" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D27" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E27" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F27" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G27" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H27" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I27" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1855,28 +1867,28 @@
         <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C28" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D28" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E28" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="F28" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G28" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H28" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I28" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1884,28 +1896,28 @@
         <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C29" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D29" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E29" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F29" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G29" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="H29" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I29" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1913,28 +1925,28 @@
         <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C30" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D30" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E30" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F30" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G30" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="H30" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I30" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1942,28 +1954,28 @@
         <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C31" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D31" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E31" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F31" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G31" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="H31" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I31" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1971,28 +1983,28 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C32" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D32" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E32" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F32" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G32" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="H32" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I32" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -2000,28 +2012,28 @@
         <v>40</v>
       </c>
       <c r="B33" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C33" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D33" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E33" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F33" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G33" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="H33" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I33" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -2029,28 +2041,28 @@
         <v>41</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C34" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D34" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E34" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="F34" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G34" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="H34" t="s">
-        <v>240</v>
+        <v>244</v>
       </c>
       <c r="I34" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -2058,28 +2070,28 @@
         <v>42</v>
       </c>
       <c r="B35" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C35" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D35" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E35" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F35" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G35" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H35" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I35" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -2087,28 +2099,28 @@
         <v>43</v>
       </c>
       <c r="B36" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C36" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D36" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E36" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F36" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G36" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H36" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I36" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -2116,28 +2128,28 @@
         <v>44</v>
       </c>
       <c r="B37" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D37" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E37" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F37" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G37" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H37" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I37" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -2145,28 +2157,28 @@
         <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D38" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E38" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F38" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G38" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H38" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I38" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -2174,28 +2186,28 @@
         <v>46</v>
       </c>
       <c r="B39" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C39" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D39" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E39" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F39" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G39" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H39" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I39" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2203,28 +2215,28 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C40" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D40" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E40" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F40" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G40" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H40" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I40" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2232,28 +2244,28 @@
         <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C41" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D41" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E41" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F41" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G41" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H41" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I41" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2261,28 +2273,28 @@
         <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C42" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D42" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E42" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="F42" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G42" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H42" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I42" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -2290,28 +2302,28 @@
         <v>50</v>
       </c>
       <c r="B43" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C43" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D43" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E43" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F43" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G43" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H43" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I43" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -2319,28 +2331,28 @@
         <v>51</v>
       </c>
       <c r="B44" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C44" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D44" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E44" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F44" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G44" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H44" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I44" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -2348,28 +2360,28 @@
         <v>52</v>
       </c>
       <c r="B45" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C45" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D45" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E45" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F45" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G45" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H45" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I45" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -2377,28 +2389,28 @@
         <v>53</v>
       </c>
       <c r="B46" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C46" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D46" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E46" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F46" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G46" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H46" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I46" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -2406,28 +2418,28 @@
         <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C47" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D47" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E47" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F47" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G47" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H47" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I47" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -2435,28 +2447,28 @@
         <v>55</v>
       </c>
       <c r="B48" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C48" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D48" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E48" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F48" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G48" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H48" t="s">
-        <v>239</v>
+        <v>243</v>
       </c>
       <c r="I48" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -2464,19 +2476,19 @@
         <v>56</v>
       </c>
       <c r="B49" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C49" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F49" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="H49" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I49" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2484,22 +2496,22 @@
         <v>57</v>
       </c>
       <c r="B50" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C50" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F50" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G50" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="H50" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I50" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2507,19 +2519,19 @@
         <v>58</v>
       </c>
       <c r="B51" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C51" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F51" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="H51" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I51" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2527,22 +2539,22 @@
         <v>59</v>
       </c>
       <c r="B52" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C52" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E52" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F52" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="H52" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I52" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2550,22 +2562,22 @@
         <v>60</v>
       </c>
       <c r="B53" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C53" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E53" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F53" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="H53" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I53" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2573,22 +2585,22 @@
         <v>61</v>
       </c>
       <c r="B54" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C54" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F54" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G54" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="H54" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I54" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2596,28 +2608,28 @@
         <v>62</v>
       </c>
       <c r="B55" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C55" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="D55" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E55" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F55" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G55" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H55" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I55" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2625,28 +2637,28 @@
         <v>63</v>
       </c>
       <c r="B56" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C56" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D56" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E56" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F56" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G56" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H56" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I56" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2654,28 +2666,28 @@
         <v>64</v>
       </c>
       <c r="B57" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C57" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D57" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E57" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F57" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G57" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H57" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I57" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2683,28 +2695,28 @@
         <v>65</v>
       </c>
       <c r="B58" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C58" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D58" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E58" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F58" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G58" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H58" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I58" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2712,28 +2724,28 @@
         <v>66</v>
       </c>
       <c r="B59" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C59" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D59" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E59" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F59" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G59" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H59" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I59" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2741,28 +2753,28 @@
         <v>67</v>
       </c>
       <c r="B60" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C60" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D60" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E60" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="F60" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G60" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H60" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I60" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2770,28 +2782,28 @@
         <v>68</v>
       </c>
       <c r="B61" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C61" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D61" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E61" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F61" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G61" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H61" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I61" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2799,28 +2811,28 @@
         <v>69</v>
       </c>
       <c r="B62" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C62" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D62" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E62" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F62" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G62" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H62" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I62" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2828,28 +2840,28 @@
         <v>70</v>
       </c>
       <c r="B63" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C63" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D63" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E63" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F63" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G63" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H63" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I63" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2857,28 +2869,28 @@
         <v>71</v>
       </c>
       <c r="B64" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C64" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D64" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E64" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F64" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G64" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H64" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I64" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2886,28 +2898,28 @@
         <v>72</v>
       </c>
       <c r="B65" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C65" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D65" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E65" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F65" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G65" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H65" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I65" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -2915,25 +2927,25 @@
         <v>73</v>
       </c>
       <c r="B66" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C66" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D66" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F66" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G66" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H66" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I66" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -2941,25 +2953,25 @@
         <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C67" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D67" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F67" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G67" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H67" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I67" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -2967,28 +2979,28 @@
         <v>75</v>
       </c>
       <c r="B68" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C68" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D68" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E68" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F68" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G68" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H68" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I68" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -2996,28 +3008,28 @@
         <v>76</v>
       </c>
       <c r="B69" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C69" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D69" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E69" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F69" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G69" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H69" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I69" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3025,28 +3037,28 @@
         <v>77</v>
       </c>
       <c r="B70" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C70" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D70" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E70" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F70" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G70" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H70" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I70" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -3054,28 +3066,28 @@
         <v>78</v>
       </c>
       <c r="B71" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C71" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D71" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E71" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="F71" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G71" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H71" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I71" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -3083,28 +3095,28 @@
         <v>79</v>
       </c>
       <c r="B72" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C72" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D72" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E72" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F72" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G72" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H72" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I72" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -3112,28 +3124,28 @@
         <v>80</v>
       </c>
       <c r="B73" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C73" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D73" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E73" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F73" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G73" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H73" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I73" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -3141,28 +3153,28 @@
         <v>81</v>
       </c>
       <c r="B74" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C74" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D74" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E74" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F74" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G74" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H74" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I74" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3170,28 +3182,28 @@
         <v>82</v>
       </c>
       <c r="B75" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C75" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D75" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E75" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F75" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G75" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H75" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I75" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3199,28 +3211,28 @@
         <v>83</v>
       </c>
       <c r="B76" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C76" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D76" t="s">
+        <v>154</v>
+      </c>
+      <c r="E76" t="s">
+        <v>227</v>
+      </c>
+      <c r="F76" t="s">
+        <v>236</v>
+      </c>
+      <c r="G76" t="s">
         <v>152</v>
       </c>
-      <c r="E76" t="s">
-        <v>224</v>
-      </c>
-      <c r="F76" t="s">
-        <v>232</v>
-      </c>
-      <c r="G76" t="s">
-        <v>151</v>
-      </c>
       <c r="H76" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I76" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3228,22 +3240,22 @@
         <v>84</v>
       </c>
       <c r="B77" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C77" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E77" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F77" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="H77" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I77" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3251,28 +3263,28 @@
         <v>85</v>
       </c>
       <c r="B78" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C78" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D78" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E78" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F78" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G78" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H78" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I78" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3280,28 +3292,28 @@
         <v>86</v>
       </c>
       <c r="B79" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C79" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D79" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="E79" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F79" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G79" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H79" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I79" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3309,28 +3321,28 @@
         <v>87</v>
       </c>
       <c r="B80" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C80" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D80" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E80" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F80" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G80" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H80" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I80" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3338,28 +3350,28 @@
         <v>88</v>
       </c>
       <c r="B81" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C81" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D81" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E81" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F81" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G81" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H81" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I81" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3367,28 +3379,28 @@
         <v>89</v>
       </c>
       <c r="B82" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C82" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D82" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E82" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F82" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="G82" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H82" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="I82" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3396,28 +3408,57 @@
         <v>90</v>
       </c>
       <c r="B83" t="s">
+        <v>128</v>
+      </c>
+      <c r="C83" t="s">
+        <v>136</v>
+      </c>
+      <c r="D83" t="s">
+        <v>157</v>
+      </c>
+      <c r="E83" t="s">
+        <v>234</v>
+      </c>
+      <c r="F83" t="s">
+        <v>236</v>
+      </c>
+      <c r="G83" t="s">
+        <v>136</v>
+      </c>
+      <c r="H83" t="s">
+        <v>242</v>
+      </c>
+      <c r="I83" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" t="s">
+        <v>91</v>
+      </c>
+      <c r="B84" t="s">
         <v>127</v>
       </c>
-      <c r="C83" t="s">
-        <v>135</v>
-      </c>
-      <c r="D83" t="s">
-        <v>155</v>
-      </c>
-      <c r="E83" t="s">
-        <v>231</v>
-      </c>
-      <c r="F83" t="s">
-        <v>232</v>
-      </c>
-      <c r="G83" t="s">
-        <v>135</v>
-      </c>
-      <c r="H83" t="s">
-        <v>238</v>
-      </c>
-      <c r="I83" t="s">
-        <v>241</v>
+      <c r="C84" t="s">
+        <v>153</v>
+      </c>
+      <c r="D84" t="s">
+        <v>163</v>
+      </c>
+      <c r="E84" t="s">
+        <v>235</v>
+      </c>
+      <c r="F84" t="s">
+        <v>236</v>
+      </c>
+      <c r="G84" t="s">
+        <v>153</v>
+      </c>
+      <c r="H84" t="s">
+        <v>242</v>
+      </c>
+      <c r="I84" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
sync: actualizar catálogo maestro de POs con INT-0071 (PO 2609-3665)
</commit_message>
<xml_diff>
--- a/BD_POs_Cabecera.xlsx
+++ b/BD_POs_Cabecera.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="249">
   <si>
     <t>PO</t>
   </si>
@@ -292,6 +292,9 @@
     <t>26093636</t>
   </si>
   <si>
+    <t>26093665</t>
+  </si>
+  <si>
     <t>2026-08-17</t>
   </si>
   <si>
@@ -403,6 +406,9 @@
     <t>2026-09-07</t>
   </si>
   <si>
+    <t>2026-09-09</t>
+  </si>
+  <si>
     <t>CLOUD</t>
   </si>
   <si>
@@ -722,6 +728,9 @@
   </si>
   <si>
     <t>23489, 23495, 23264</t>
+  </si>
+  <si>
+    <t>23203</t>
   </si>
   <si>
     <t>ALMACEN SIGRAMA</t>
@@ -1085,7 +1094,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I84"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -1122,28 +1131,28 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C2" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F2" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G2" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="H2" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I2" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1151,28 +1160,28 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F3" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H3" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I3" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1180,25 +1189,25 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="D4" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F4" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G4" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H4" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I4" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1206,28 +1215,28 @@
         <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="E5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F5" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H5" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I5" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1235,28 +1244,28 @@
         <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D6" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F6" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H6" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I6" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1264,28 +1273,28 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D7" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E7" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F7" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G7" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H7" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I7" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1293,28 +1302,28 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D8" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E8" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F8" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H8" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I8" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1322,28 +1331,28 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D9" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G9" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1351,28 +1360,28 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C10" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D10" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E10" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F10" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G10" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="H10" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I10" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1380,28 +1389,28 @@
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D11" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E11" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F11" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G11" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H11" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I11" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1409,28 +1418,28 @@
         <v>19</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D12" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E12" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F12" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H12" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I12" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1438,25 +1447,25 @@
         <v>20</v>
       </c>
       <c r="B13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="D13" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F13" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G13" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H13" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I13" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1464,28 +1473,28 @@
         <v>21</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C14" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D14" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E14" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F14" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G14" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H14" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I14" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1493,28 +1502,28 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D15" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E15" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F15" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H15" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I15" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1522,28 +1531,28 @@
         <v>23</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D16" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F16" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G16" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H16" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I16" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1551,28 +1560,28 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C17" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D17" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E17" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F17" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G17" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H17" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I17" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1580,28 +1589,28 @@
         <v>25</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C18" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D18" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E18" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F18" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G18" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H18" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I18" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1609,28 +1618,28 @@
         <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C19" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D19" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E19" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="F19" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G19" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H19" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I19" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1638,25 +1647,25 @@
         <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C20" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D20" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F20" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G20" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H20" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I20" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1664,28 +1673,28 @@
         <v>28</v>
       </c>
       <c r="B21" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D21" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E21" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F21" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G21" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H21" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I21" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1693,28 +1702,28 @@
         <v>29</v>
       </c>
       <c r="B22" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C22" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D22" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E22" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F22" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G22" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H22" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I22" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1722,28 +1731,28 @@
         <v>30</v>
       </c>
       <c r="B23" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C23" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E23" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F23" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G23" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H23" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I23" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1751,28 +1760,28 @@
         <v>31</v>
       </c>
       <c r="B24" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C24" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D24" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E24" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="F24" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G24" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H24" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I24" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1780,28 +1789,28 @@
         <v>32</v>
       </c>
       <c r="B25" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C25" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D25" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E25" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F25" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G25" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H25" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I25" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1809,28 +1818,28 @@
         <v>33</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C26" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D26" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E26" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F26" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G26" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H26" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I26" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1838,28 +1847,28 @@
         <v>34</v>
       </c>
       <c r="B27" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C27" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D27" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E27" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="F27" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G27" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H27" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I27" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1867,28 +1876,28 @@
         <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C28" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D28" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E28" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F28" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G28" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H28" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I28" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1896,28 +1905,28 @@
         <v>36</v>
       </c>
       <c r="B29" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C29" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D29" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E29" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F29" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G29" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H29" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="I29" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1925,28 +1934,28 @@
         <v>37</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D30" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E30" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="F30" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G30" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H30" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="I30" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1954,28 +1963,28 @@
         <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C31" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D31" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E31" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F31" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G31" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H31" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="I31" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -1983,28 +1992,28 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C32" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D32" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E32" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="F32" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G32" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H32" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="I32" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -2012,28 +2021,28 @@
         <v>40</v>
       </c>
       <c r="B33" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C33" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D33" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E33" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F33" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G33" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H33" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="I33" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -2041,28 +2050,28 @@
         <v>41</v>
       </c>
       <c r="B34" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C34" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D34" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E34" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F34" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G34" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="H34" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="I34" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -2070,28 +2079,28 @@
         <v>42</v>
       </c>
       <c r="B35" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C35" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D35" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E35" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="F35" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G35" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H35" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I35" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -2099,28 +2108,28 @@
         <v>43</v>
       </c>
       <c r="B36" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C36" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E36" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="F36" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G36" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H36" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I36" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -2128,28 +2137,28 @@
         <v>44</v>
       </c>
       <c r="B37" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C37" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D37" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E37" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F37" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G37" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H37" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I37" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -2157,28 +2166,28 @@
         <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C38" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E38" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F38" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G38" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H38" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I38" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -2186,28 +2195,28 @@
         <v>46</v>
       </c>
       <c r="B39" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C39" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D39" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E39" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F39" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G39" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H39" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I39" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2215,28 +2224,28 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C40" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D40" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E40" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F40" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G40" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H40" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I40" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2244,28 +2253,28 @@
         <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C41" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D41" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E41" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F41" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G41" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H41" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I41" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2273,28 +2282,28 @@
         <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C42" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D42" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E42" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="F42" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G42" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H42" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I42" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -2302,28 +2311,28 @@
         <v>50</v>
       </c>
       <c r="B43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C43" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E43" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F43" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G43" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H43" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I43" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -2331,28 +2340,28 @@
         <v>51</v>
       </c>
       <c r="B44" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C44" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D44" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E44" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="F44" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G44" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H44" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I44" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -2360,28 +2369,28 @@
         <v>52</v>
       </c>
       <c r="B45" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C45" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D45" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E45" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F45" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G45" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H45" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I45" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -2389,28 +2398,28 @@
         <v>53</v>
       </c>
       <c r="B46" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C46" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D46" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E46" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F46" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G46" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H46" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I46" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -2418,28 +2427,28 @@
         <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C47" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E47" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F47" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G47" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H47" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I47" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -2447,28 +2456,28 @@
         <v>55</v>
       </c>
       <c r="B48" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C48" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D48" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E48" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F48" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G48" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="H48" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I48" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -2476,19 +2485,19 @@
         <v>56</v>
       </c>
       <c r="B49" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C49" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F49" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="H49" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I49" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2496,22 +2505,22 @@
         <v>57</v>
       </c>
       <c r="B50" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C50" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F50" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G50" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="H50" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I50" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2519,19 +2528,19 @@
         <v>58</v>
       </c>
       <c r="B51" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C51" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F51" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="H51" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I51" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2539,22 +2548,22 @@
         <v>59</v>
       </c>
       <c r="B52" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C52" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E52" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F52" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="H52" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I52" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2562,22 +2571,22 @@
         <v>60</v>
       </c>
       <c r="B53" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C53" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E53" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F53" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="H53" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I53" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2585,22 +2594,22 @@
         <v>61</v>
       </c>
       <c r="B54" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C54" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F54" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G54" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="H54" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I54" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2608,28 +2617,28 @@
         <v>62</v>
       </c>
       <c r="B55" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C55" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D55" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E55" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="F55" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G55" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="H55" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I55" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2637,28 +2646,28 @@
         <v>63</v>
       </c>
       <c r="B56" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C56" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D56" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E56" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F56" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G56" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H56" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I56" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2666,28 +2675,28 @@
         <v>64</v>
       </c>
       <c r="B57" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C57" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D57" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E57" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="F57" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G57" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H57" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I57" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2695,28 +2704,28 @@
         <v>65</v>
       </c>
       <c r="B58" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C58" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D58" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E58" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F58" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G58" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H58" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I58" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2724,28 +2733,28 @@
         <v>66</v>
       </c>
       <c r="B59" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C59" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D59" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E59" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="F59" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G59" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H59" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I59" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2753,28 +2762,28 @@
         <v>67</v>
       </c>
       <c r="B60" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C60" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D60" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E60" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F60" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G60" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H60" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I60" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2782,28 +2791,28 @@
         <v>68</v>
       </c>
       <c r="B61" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C61" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D61" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E61" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F61" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G61" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H61" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I61" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2811,28 +2820,28 @@
         <v>69</v>
       </c>
       <c r="B62" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C62" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D62" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E62" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F62" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G62" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H62" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I62" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2840,28 +2849,28 @@
         <v>70</v>
       </c>
       <c r="B63" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C63" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D63" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E63" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F63" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G63" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H63" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I63" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2869,28 +2878,28 @@
         <v>71</v>
       </c>
       <c r="B64" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C64" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D64" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E64" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F64" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G64" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H64" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I64" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2898,28 +2907,28 @@
         <v>72</v>
       </c>
       <c r="B65" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C65" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D65" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E65" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F65" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G65" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H65" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I65" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -2927,25 +2936,25 @@
         <v>73</v>
       </c>
       <c r="B66" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C66" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D66" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F66" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G66" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H66" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I66" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -2953,25 +2962,25 @@
         <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C67" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D67" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F67" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G67" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H67" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I67" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -2979,28 +2988,28 @@
         <v>75</v>
       </c>
       <c r="B68" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C68" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D68" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E68" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F68" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G68" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H68" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I68" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -3008,28 +3017,28 @@
         <v>76</v>
       </c>
       <c r="B69" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C69" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D69" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E69" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F69" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G69" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H69" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I69" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3037,28 +3046,28 @@
         <v>77</v>
       </c>
       <c r="B70" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C70" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D70" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E70" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F70" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G70" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H70" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I70" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -3066,28 +3075,28 @@
         <v>78</v>
       </c>
       <c r="B71" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C71" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D71" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E71" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F71" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G71" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H71" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I71" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -3095,28 +3104,28 @@
         <v>79</v>
       </c>
       <c r="B72" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C72" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D72" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="E72" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="F72" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G72" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H72" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I72" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -3124,28 +3133,28 @@
         <v>80</v>
       </c>
       <c r="B73" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D73" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E73" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F73" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G73" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H73" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I73" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -3153,28 +3162,28 @@
         <v>81</v>
       </c>
       <c r="B74" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C74" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D74" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E74" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F74" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G74" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H74" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I74" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3182,28 +3191,28 @@
         <v>82</v>
       </c>
       <c r="B75" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C75" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D75" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E75" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="F75" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G75" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H75" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I75" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3211,28 +3220,28 @@
         <v>83</v>
       </c>
       <c r="B76" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C76" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D76" t="s">
+        <v>156</v>
+      </c>
+      <c r="E76" t="s">
+        <v>229</v>
+      </c>
+      <c r="F76" t="s">
+        <v>239</v>
+      </c>
+      <c r="G76" t="s">
         <v>154</v>
       </c>
-      <c r="E76" t="s">
-        <v>227</v>
-      </c>
-      <c r="F76" t="s">
-        <v>236</v>
-      </c>
-      <c r="G76" t="s">
-        <v>152</v>
-      </c>
       <c r="H76" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I76" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3240,22 +3249,22 @@
         <v>84</v>
       </c>
       <c r="B77" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C77" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="E77" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="F77" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="H77" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I77" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3263,28 +3272,28 @@
         <v>85</v>
       </c>
       <c r="B78" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C78" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D78" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="E78" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F78" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G78" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H78" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I78" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3292,28 +3301,28 @@
         <v>86</v>
       </c>
       <c r="B79" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C79" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D79" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="E79" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F79" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G79" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H79" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I79" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3321,28 +3330,28 @@
         <v>87</v>
       </c>
       <c r="B80" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C80" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D80" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E80" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="F80" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G80" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H80" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I80" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3350,28 +3359,28 @@
         <v>88</v>
       </c>
       <c r="B81" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C81" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D81" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E81" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="F81" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G81" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H81" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I81" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3379,28 +3388,28 @@
         <v>89</v>
       </c>
       <c r="B82" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C82" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D82" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="E82" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F82" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G82" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H82" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I82" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3408,28 +3417,28 @@
         <v>90</v>
       </c>
       <c r="B83" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C83" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="D83" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="E83" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F83" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G83" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H83" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I83" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -3437,28 +3446,57 @@
         <v>91</v>
       </c>
       <c r="B84" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C84" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D84" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E84" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F84" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="G84" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H84" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="I84" t="s">
-        <v>245</v>
+        <v>248</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" t="s">
+        <v>92</v>
+      </c>
+      <c r="B85" t="s">
+        <v>130</v>
+      </c>
+      <c r="C85" t="s">
+        <v>131</v>
+      </c>
+      <c r="D85" t="s">
+        <v>156</v>
+      </c>
+      <c r="E85" t="s">
+        <v>238</v>
+      </c>
+      <c r="F85" t="s">
+        <v>239</v>
+      </c>
+      <c r="G85" t="s">
+        <v>131</v>
+      </c>
+      <c r="H85" t="s">
+        <v>245</v>
+      </c>
+      <c r="I85" t="s">
+        <v>248</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sincronizar BD_POs_Cabecera y Requerimientos con entregas historicas 100%
</commit_message>
<xml_diff>
--- a/BD_POs_Cabecera.xlsx
+++ b/BD_POs_Cabecera.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="250">
   <si>
     <t>PO</t>
   </si>
@@ -760,6 +760,9 @@
   </si>
   <si>
     <t>#EF4444</t>
+  </si>
+  <si>
+    <t>#10B981</t>
   </si>
   <si>
     <t>#FFFFFF</t>
@@ -1152,7 +1155,7 @@
         <v>245</v>
       </c>
       <c r="I2" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1181,7 +1184,7 @@
         <v>245</v>
       </c>
       <c r="I3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1207,7 +1210,7 @@
         <v>245</v>
       </c>
       <c r="I4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1236,7 +1239,7 @@
         <v>245</v>
       </c>
       <c r="I5" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1265,7 +1268,7 @@
         <v>245</v>
       </c>
       <c r="I6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1294,7 +1297,7 @@
         <v>245</v>
       </c>
       <c r="I7" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1323,7 +1326,7 @@
         <v>245</v>
       </c>
       <c r="I8" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1352,7 +1355,7 @@
         <v>245</v>
       </c>
       <c r="I9" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1381,7 +1384,7 @@
         <v>245</v>
       </c>
       <c r="I10" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1410,7 +1413,7 @@
         <v>245</v>
       </c>
       <c r="I11" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1439,7 +1442,7 @@
         <v>245</v>
       </c>
       <c r="I12" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1465,7 +1468,7 @@
         <v>245</v>
       </c>
       <c r="I13" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1494,7 +1497,7 @@
         <v>245</v>
       </c>
       <c r="I14" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1523,7 +1526,7 @@
         <v>245</v>
       </c>
       <c r="I15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1552,7 +1555,7 @@
         <v>245</v>
       </c>
       <c r="I16" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1581,7 +1584,7 @@
         <v>245</v>
       </c>
       <c r="I17" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1610,7 +1613,7 @@
         <v>245</v>
       </c>
       <c r="I18" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1639,7 +1642,7 @@
         <v>245</v>
       </c>
       <c r="I19" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1665,7 +1668,7 @@
         <v>246</v>
       </c>
       <c r="I20" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1694,7 +1697,7 @@
         <v>245</v>
       </c>
       <c r="I21" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1723,7 +1726,7 @@
         <v>245</v>
       </c>
       <c r="I22" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1752,7 +1755,7 @@
         <v>245</v>
       </c>
       <c r="I23" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1781,7 +1784,7 @@
         <v>245</v>
       </c>
       <c r="I24" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1810,7 +1813,7 @@
         <v>245</v>
       </c>
       <c r="I25" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1839,7 +1842,7 @@
         <v>245</v>
       </c>
       <c r="I26" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1868,7 +1871,7 @@
         <v>245</v>
       </c>
       <c r="I27" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1897,7 +1900,7 @@
         <v>246</v>
       </c>
       <c r="I28" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1926,7 +1929,7 @@
         <v>247</v>
       </c>
       <c r="I29" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1955,7 +1958,7 @@
         <v>247</v>
       </c>
       <c r="I30" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1984,7 +1987,7 @@
         <v>247</v>
       </c>
       <c r="I31" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -2013,7 +2016,7 @@
         <v>247</v>
       </c>
       <c r="I32" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -2042,7 +2045,7 @@
         <v>247</v>
       </c>
       <c r="I33" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -2071,7 +2074,7 @@
         <v>247</v>
       </c>
       <c r="I34" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -2100,7 +2103,7 @@
         <v>246</v>
       </c>
       <c r="I35" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -2129,7 +2132,7 @@
         <v>246</v>
       </c>
       <c r="I36" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -2158,7 +2161,7 @@
         <v>246</v>
       </c>
       <c r="I37" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -2187,7 +2190,7 @@
         <v>246</v>
       </c>
       <c r="I38" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -2216,7 +2219,7 @@
         <v>246</v>
       </c>
       <c r="I39" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2245,7 +2248,7 @@
         <v>246</v>
       </c>
       <c r="I40" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2274,7 +2277,7 @@
         <v>246</v>
       </c>
       <c r="I41" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2303,7 +2306,7 @@
         <v>246</v>
       </c>
       <c r="I42" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -2332,7 +2335,7 @@
         <v>246</v>
       </c>
       <c r="I43" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -2361,7 +2364,7 @@
         <v>246</v>
       </c>
       <c r="I44" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -2390,7 +2393,7 @@
         <v>246</v>
       </c>
       <c r="I45" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -2419,7 +2422,7 @@
         <v>246</v>
       </c>
       <c r="I46" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -2448,7 +2451,7 @@
         <v>246</v>
       </c>
       <c r="I47" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -2477,7 +2480,7 @@
         <v>246</v>
       </c>
       <c r="I48" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -2494,10 +2497,10 @@
         <v>239</v>
       </c>
       <c r="H49" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I49" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2520,7 +2523,7 @@
         <v>245</v>
       </c>
       <c r="I50" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2540,7 +2543,7 @@
         <v>245</v>
       </c>
       <c r="I51" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2563,7 +2566,7 @@
         <v>245</v>
       </c>
       <c r="I52" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2586,7 +2589,7 @@
         <v>245</v>
       </c>
       <c r="I53" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2609,7 +2612,7 @@
         <v>245</v>
       </c>
       <c r="I54" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2638,7 +2641,7 @@
         <v>245</v>
       </c>
       <c r="I55" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2667,7 +2670,7 @@
         <v>245</v>
       </c>
       <c r="I56" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2693,10 +2696,10 @@
         <v>145</v>
       </c>
       <c r="H57" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I57" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2722,10 +2725,10 @@
         <v>145</v>
       </c>
       <c r="H58" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I58" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2754,7 +2757,7 @@
         <v>245</v>
       </c>
       <c r="I59" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2783,7 +2786,7 @@
         <v>245</v>
       </c>
       <c r="I60" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2809,10 +2812,10 @@
         <v>147</v>
       </c>
       <c r="H61" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I61" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2838,10 +2841,10 @@
         <v>148</v>
       </c>
       <c r="H62" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I62" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2867,10 +2870,10 @@
         <v>134</v>
       </c>
       <c r="H63" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I63" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2896,10 +2899,10 @@
         <v>149</v>
       </c>
       <c r="H64" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I64" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2925,10 +2928,10 @@
         <v>150</v>
       </c>
       <c r="H65" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I65" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -2951,10 +2954,10 @@
         <v>147</v>
       </c>
       <c r="H66" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I66" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -2977,10 +2980,10 @@
         <v>146</v>
       </c>
       <c r="H67" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I67" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -3006,10 +3009,10 @@
         <v>134</v>
       </c>
       <c r="H68" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I68" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -3035,10 +3038,10 @@
         <v>144</v>
       </c>
       <c r="H69" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I69" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3064,10 +3067,10 @@
         <v>147</v>
       </c>
       <c r="H70" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I70" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -3093,10 +3096,10 @@
         <v>148</v>
       </c>
       <c r="H71" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I71" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -3125,7 +3128,7 @@
         <v>245</v>
       </c>
       <c r="I72" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -3154,7 +3157,7 @@
         <v>245</v>
       </c>
       <c r="I73" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -3183,7 +3186,7 @@
         <v>245</v>
       </c>
       <c r="I74" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3212,7 +3215,7 @@
         <v>245</v>
       </c>
       <c r="I75" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3241,7 +3244,7 @@
         <v>245</v>
       </c>
       <c r="I76" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3261,10 +3264,10 @@
         <v>239</v>
       </c>
       <c r="H77" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="I77" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3293,7 +3296,7 @@
         <v>245</v>
       </c>
       <c r="I78" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3322,7 +3325,7 @@
         <v>245</v>
       </c>
       <c r="I79" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3351,7 +3354,7 @@
         <v>245</v>
       </c>
       <c r="I80" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3380,7 +3383,7 @@
         <v>245</v>
       </c>
       <c r="I81" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3409,7 +3412,7 @@
         <v>245</v>
       </c>
       <c r="I82" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3438,7 +3441,7 @@
         <v>245</v>
       </c>
       <c r="I83" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -3467,7 +3470,7 @@
         <v>245</v>
       </c>
       <c r="I84" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -3496,7 +3499,7 @@
         <v>245</v>
       </c>
       <c r="I85" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizar proyectos de POs segun imagen maestro
</commit_message>
<xml_diff>
--- a/BD_POs_Cabecera.xlsx
+++ b/BD_POs_Cabecera.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="749" uniqueCount="235">
   <si>
     <t>PO</t>
   </si>
@@ -424,7 +424,7 @@
     <t>TORONTO</t>
   </si>
   <si>
-    <t>IRVING LK - IRVING PP</t>
+    <t>IRVING LX - IRVING PP</t>
   </si>
   <si>
     <t>RENO 6</t>
@@ -445,45 +445,12 @@
     <t>SIGRAMA LASER</t>
   </si>
   <si>
-    <t>RENO4 CDC582</t>
-  </si>
-  <si>
-    <t>ALM LC8 CDC 672</t>
-  </si>
-  <si>
-    <t>ALM LC8 CDC 672 20K</t>
-  </si>
-  <si>
-    <t>SWBD R4</t>
-  </si>
-  <si>
-    <t>SWBD R5</t>
-  </si>
-  <si>
-    <t>SWBD R6</t>
-  </si>
-  <si>
-    <t>ALM RENO 5 CDC 557</t>
-  </si>
-  <si>
-    <t>LC8 CLOUD</t>
-  </si>
-  <si>
     <t>LC8 20 K</t>
   </si>
   <si>
-    <t>CC 707 CE 1852-TAB</t>
-  </si>
-  <si>
     <t>SOUTH VALLEY</t>
   </si>
   <si>
-    <t>SWBD RENO 4</t>
-  </si>
-  <si>
-    <t>SWBDLC8</t>
-  </si>
-  <si>
     <t>ESTEFANIA IBARRA</t>
   </si>
   <si>
@@ -736,21 +703,7 @@
     <t>ALMACEN SIGRAMA</t>
   </si>
   <si>
-    <t>ALM SWBD CDC 736</t>
-  </si>
-  <si>
-    <t>CC707 CE 1852-TAB</t>
-  </si>
-  <si>
-    <t>REGISTRADA</t>
-  </si>
-  <si>
     <t>CANCELADO</t>
-  </si>
-  <si>
-    <t>DIA
-MES
-AÑO</t>
   </si>
   <si>
     <t>#EC2024</t>
@@ -1140,22 +1093,22 @@
         <v>131</v>
       </c>
       <c r="D2" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E2" t="s">
-        <v>166</v>
+        <v>155</v>
       </c>
       <c r="F2" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G2" t="s">
-        <v>240</v>
+        <v>131</v>
       </c>
       <c r="H2" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I2" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" spans="1:9">
@@ -1169,22 +1122,22 @@
         <v>131</v>
       </c>
       <c r="D3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E3" t="s">
         <v>156</v>
       </c>
-      <c r="E3" t="s">
-        <v>167</v>
-      </c>
       <c r="F3" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G3" t="s">
         <v>131</v>
       </c>
       <c r="H3" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I3" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" spans="1:9">
@@ -1198,19 +1151,19 @@
         <v>132</v>
       </c>
       <c r="D4" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="F4" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G4" t="s">
         <v>132</v>
       </c>
       <c r="H4" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I4" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="5" spans="1:9">
@@ -1224,22 +1177,22 @@
         <v>131</v>
       </c>
       <c r="D5" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="E5" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="F5" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G5" t="s">
         <v>131</v>
       </c>
       <c r="H5" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I5" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -1253,22 +1206,22 @@
         <v>133</v>
       </c>
       <c r="D6" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E6" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="F6" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G6" t="s">
         <v>133</v>
       </c>
       <c r="H6" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I6" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="1:9">
@@ -1282,22 +1235,22 @@
         <v>131</v>
       </c>
       <c r="D7" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E7" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="F7" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G7" t="s">
         <v>131</v>
       </c>
       <c r="H7" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I7" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -1311,22 +1264,22 @@
         <v>134</v>
       </c>
       <c r="D8" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E8" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="F8" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G8" t="s">
         <v>134</v>
       </c>
       <c r="H8" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I8" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -1340,22 +1293,22 @@
         <v>135</v>
       </c>
       <c r="D9" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E9" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="F9" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G9" t="s">
         <v>135</v>
       </c>
       <c r="H9" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I9" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -1369,22 +1322,22 @@
         <v>131</v>
       </c>
       <c r="D10" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E10" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="F10" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G10" t="s">
-        <v>240</v>
+        <v>131</v>
       </c>
       <c r="H10" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I10" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -1398,22 +1351,22 @@
         <v>133</v>
       </c>
       <c r="D11" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E11" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="F11" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G11" t="s">
         <v>133</v>
       </c>
       <c r="H11" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I11" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -1427,22 +1380,22 @@
         <v>133</v>
       </c>
       <c r="D12" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E12" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="F12" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G12" t="s">
         <v>133</v>
       </c>
       <c r="H12" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I12" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="13" spans="1:9">
@@ -1456,19 +1409,19 @@
         <v>136</v>
       </c>
       <c r="D13" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="F13" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G13" t="s">
         <v>136</v>
       </c>
       <c r="H13" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I13" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -1482,22 +1435,22 @@
         <v>137</v>
       </c>
       <c r="D14" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E14" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="F14" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G14" t="s">
         <v>137</v>
       </c>
       <c r="H14" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I14" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="15" spans="1:9">
@@ -1511,22 +1464,22 @@
         <v>137</v>
       </c>
       <c r="D15" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E15" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="F15" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G15" t="s">
         <v>137</v>
       </c>
       <c r="H15" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I15" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="16" spans="1:9">
@@ -1540,22 +1493,22 @@
         <v>137</v>
       </c>
       <c r="D16" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E16" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="F16" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G16" t="s">
         <v>137</v>
       </c>
       <c r="H16" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I16" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -1569,22 +1522,22 @@
         <v>133</v>
       </c>
       <c r="D17" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E17" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="F17" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G17" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H17" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I17" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -1598,22 +1551,22 @@
         <v>133</v>
       </c>
       <c r="D18" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E18" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="F18" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G18" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H18" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I18" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -1627,22 +1580,22 @@
         <v>133</v>
       </c>
       <c r="D19" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E19" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="F19" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G19" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H19" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I19" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1656,19 +1609,19 @@
         <v>133</v>
       </c>
       <c r="D20" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="F20" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G20" t="s">
-        <v>242</v>
+        <v>133</v>
       </c>
       <c r="H20" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I20" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="21" spans="1:9">
@@ -1682,22 +1635,22 @@
         <v>133</v>
       </c>
       <c r="D21" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E21" t="s">
-        <v>181</v>
+        <v>170</v>
       </c>
       <c r="F21" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G21" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H21" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I21" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1711,22 +1664,22 @@
         <v>133</v>
       </c>
       <c r="D22" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E22" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="F22" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G22" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H22" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I22" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -1740,22 +1693,22 @@
         <v>133</v>
       </c>
       <c r="D23" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E23" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="F23" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G23" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H23" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I23" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1769,22 +1722,22 @@
         <v>133</v>
       </c>
       <c r="D24" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E24" t="s">
-        <v>184</v>
+        <v>173</v>
       </c>
       <c r="F24" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G24" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H24" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I24" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1798,22 +1751,22 @@
         <v>133</v>
       </c>
       <c r="D25" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E25" t="s">
-        <v>185</v>
+        <v>174</v>
       </c>
       <c r="F25" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G25" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H25" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I25" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="26" spans="1:9">
@@ -1827,22 +1780,22 @@
         <v>133</v>
       </c>
       <c r="D26" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E26" t="s">
-        <v>186</v>
+        <v>175</v>
       </c>
       <c r="F26" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G26" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H26" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I26" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -1856,22 +1809,22 @@
         <v>133</v>
       </c>
       <c r="D27" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E27" t="s">
-        <v>187</v>
+        <v>176</v>
       </c>
       <c r="F27" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G27" t="s">
-        <v>241</v>
+        <v>133</v>
       </c>
       <c r="H27" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I27" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="28" spans="1:9">
@@ -1885,22 +1838,22 @@
         <v>137</v>
       </c>
       <c r="D28" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E28" t="s">
-        <v>188</v>
+        <v>177</v>
       </c>
       <c r="F28" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G28" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H28" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I28" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="29" spans="1:9">
@@ -1914,22 +1867,22 @@
         <v>138</v>
       </c>
       <c r="D29" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E29" t="s">
-        <v>189</v>
+        <v>178</v>
       </c>
       <c r="F29" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G29" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H29" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="I29" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="30" spans="1:9">
@@ -1943,22 +1896,22 @@
         <v>138</v>
       </c>
       <c r="D30" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E30" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="F30" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G30" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H30" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="I30" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="31" spans="1:9">
@@ -1972,22 +1925,22 @@
         <v>138</v>
       </c>
       <c r="D31" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E31" t="s">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="F31" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G31" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H31" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="I31" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:9">
@@ -2001,22 +1954,22 @@
         <v>138</v>
       </c>
       <c r="D32" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E32" t="s">
-        <v>192</v>
+        <v>181</v>
       </c>
       <c r="F32" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G32" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H32" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="I32" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="33" spans="1:9">
@@ -2030,22 +1983,22 @@
         <v>138</v>
       </c>
       <c r="D33" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E33" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="F33" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G33" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H33" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="I33" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="34" spans="1:9">
@@ -2059,22 +2012,22 @@
         <v>138</v>
       </c>
       <c r="D34" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E34" t="s">
-        <v>194</v>
+        <v>183</v>
       </c>
       <c r="F34" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G34" t="s">
-        <v>243</v>
+        <v>229</v>
       </c>
       <c r="H34" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
       <c r="I34" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="35" spans="1:9">
@@ -2088,22 +2041,22 @@
         <v>139</v>
       </c>
       <c r="D35" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E35" t="s">
-        <v>195</v>
+        <v>184</v>
       </c>
       <c r="F35" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G35" t="s">
-        <v>242</v>
+        <v>139</v>
       </c>
       <c r="H35" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I35" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="36" spans="1:9">
@@ -2117,22 +2070,22 @@
         <v>134</v>
       </c>
       <c r="D36" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E36" t="s">
-        <v>196</v>
+        <v>185</v>
       </c>
       <c r="F36" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G36" t="s">
-        <v>242</v>
+        <v>134</v>
       </c>
       <c r="H36" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I36" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="37" spans="1:9">
@@ -2146,22 +2099,22 @@
         <v>137</v>
       </c>
       <c r="D37" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E37" t="s">
-        <v>197</v>
+        <v>186</v>
       </c>
       <c r="F37" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G37" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H37" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I37" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="38" spans="1:9">
@@ -2175,22 +2128,22 @@
         <v>134</v>
       </c>
       <c r="D38" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E38" t="s">
-        <v>198</v>
+        <v>187</v>
       </c>
       <c r="F38" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G38" t="s">
-        <v>242</v>
+        <v>134</v>
       </c>
       <c r="H38" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I38" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="39" spans="1:9">
@@ -2204,22 +2157,22 @@
         <v>137</v>
       </c>
       <c r="D39" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E39" t="s">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="F39" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G39" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H39" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I39" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="40" spans="1:9">
@@ -2233,22 +2186,22 @@
         <v>137</v>
       </c>
       <c r="D40" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E40" t="s">
-        <v>200</v>
+        <v>189</v>
       </c>
       <c r="F40" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G40" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H40" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I40" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="41" spans="1:9">
@@ -2262,22 +2215,22 @@
         <v>137</v>
       </c>
       <c r="D41" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E41" t="s">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="F41" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G41" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H41" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I41" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="42" spans="1:9">
@@ -2291,22 +2244,22 @@
         <v>137</v>
       </c>
       <c r="D42" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E42" t="s">
-        <v>202</v>
+        <v>191</v>
       </c>
       <c r="F42" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G42" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H42" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I42" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="43" spans="1:9">
@@ -2320,22 +2273,22 @@
         <v>137</v>
       </c>
       <c r="D43" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E43" t="s">
-        <v>203</v>
+        <v>192</v>
       </c>
       <c r="F43" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G43" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H43" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I43" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="44" spans="1:9">
@@ -2349,22 +2302,22 @@
         <v>140</v>
       </c>
       <c r="D44" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E44" t="s">
-        <v>204</v>
+        <v>193</v>
       </c>
       <c r="F44" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G44" t="s">
-        <v>242</v>
+        <v>140</v>
       </c>
       <c r="H44" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I44" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="45" spans="1:9">
@@ -2378,22 +2331,22 @@
         <v>137</v>
       </c>
       <c r="D45" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E45" t="s">
-        <v>205</v>
+        <v>194</v>
       </c>
       <c r="F45" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G45" t="s">
-        <v>242</v>
+        <v>137</v>
       </c>
       <c r="H45" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I45" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="46" spans="1:9">
@@ -2407,22 +2360,22 @@
         <v>134</v>
       </c>
       <c r="D46" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E46" t="s">
-        <v>206</v>
+        <v>195</v>
       </c>
       <c r="F46" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G46" t="s">
-        <v>242</v>
+        <v>134</v>
       </c>
       <c r="H46" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I46" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="47" spans="1:9">
@@ -2436,22 +2389,22 @@
         <v>141</v>
       </c>
       <c r="D47" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E47" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="F47" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G47" t="s">
-        <v>242</v>
+        <v>141</v>
       </c>
       <c r="H47" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I47" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="48" spans="1:9">
@@ -2465,22 +2418,22 @@
         <v>141</v>
       </c>
       <c r="D48" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E48" t="s">
-        <v>207</v>
+        <v>196</v>
       </c>
       <c r="F48" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G48" t="s">
-        <v>242</v>
+        <v>141</v>
       </c>
       <c r="H48" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
       <c r="I48" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="49" spans="1:9">
@@ -2494,13 +2447,16 @@
         <v>139</v>
       </c>
       <c r="F49" t="s">
-        <v>239</v>
+        <v>228</v>
+      </c>
+      <c r="G49" t="s">
+        <v>139</v>
       </c>
       <c r="H49" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I49" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50" spans="1:9">
@@ -2514,16 +2470,16 @@
         <v>137</v>
       </c>
       <c r="F50" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G50" t="s">
-        <v>244</v>
+        <v>137</v>
       </c>
       <c r="H50" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I50" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="51" spans="1:9">
@@ -2537,13 +2493,16 @@
         <v>142</v>
       </c>
       <c r="F51" t="s">
-        <v>239</v>
+        <v>228</v>
+      </c>
+      <c r="G51" t="s">
+        <v>142</v>
       </c>
       <c r="H51" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I51" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="52" spans="1:9">
@@ -2557,16 +2516,19 @@
         <v>139</v>
       </c>
       <c r="E52" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
       <c r="F52" t="s">
-        <v>239</v>
+        <v>228</v>
+      </c>
+      <c r="G52" t="s">
+        <v>139</v>
       </c>
       <c r="H52" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I52" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="53" spans="1:9">
@@ -2580,16 +2542,19 @@
         <v>142</v>
       </c>
       <c r="E53" t="s">
-        <v>209</v>
+        <v>198</v>
       </c>
       <c r="F53" t="s">
-        <v>239</v>
+        <v>228</v>
+      </c>
+      <c r="G53" t="s">
+        <v>142</v>
       </c>
       <c r="H53" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I53" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="54" spans="1:9">
@@ -2603,16 +2568,16 @@
         <v>142</v>
       </c>
       <c r="F54" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G54" t="s">
-        <v>244</v>
+        <v>142</v>
       </c>
       <c r="H54" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I54" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="55" spans="1:9">
@@ -2623,25 +2588,25 @@
         <v>113</v>
       </c>
       <c r="C55" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="D55" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="E55" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
       <c r="F55" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G55" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="H55" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I55" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="56" spans="1:9">
@@ -2652,25 +2617,25 @@
         <v>109</v>
       </c>
       <c r="C56" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="D56" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="E56" t="s">
-        <v>211</v>
+        <v>200</v>
       </c>
       <c r="F56" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G56" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H56" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I56" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="57" spans="1:9">
@@ -2681,25 +2646,25 @@
         <v>114</v>
       </c>
       <c r="C57" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="D57" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E57" t="s">
-        <v>212</v>
+        <v>201</v>
       </c>
       <c r="F57" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G57" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="H57" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I57" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="58" spans="1:9">
@@ -2710,25 +2675,25 @@
         <v>114</v>
       </c>
       <c r="C58" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="D58" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E58" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
       <c r="F58" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G58" t="s">
-        <v>145</v>
+        <v>134</v>
       </c>
       <c r="H58" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I58" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="59" spans="1:9">
@@ -2739,25 +2704,25 @@
         <v>114</v>
       </c>
       <c r="C59" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D59" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E59" t="s">
-        <v>214</v>
+        <v>203</v>
       </c>
       <c r="F59" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G59" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="H59" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I59" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="60" spans="1:9">
@@ -2768,25 +2733,25 @@
         <v>114</v>
       </c>
       <c r="C60" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D60" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E60" t="s">
-        <v>215</v>
+        <v>204</v>
       </c>
       <c r="F60" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G60" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="H60" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I60" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="61" spans="1:9">
@@ -2797,25 +2762,25 @@
         <v>115</v>
       </c>
       <c r="C61" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D61" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E61" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="F61" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G61" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="H61" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I61" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="62" spans="1:9">
@@ -2826,25 +2791,25 @@
         <v>116</v>
       </c>
       <c r="C62" t="s">
+        <v>137</v>
+      </c>
+      <c r="D62" t="s">
         <v>148</v>
       </c>
-      <c r="D62" t="s">
-        <v>159</v>
-      </c>
       <c r="E62" t="s">
-        <v>217</v>
+        <v>206</v>
       </c>
       <c r="F62" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G62" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="H62" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I62" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="63" spans="1:9">
@@ -2858,22 +2823,22 @@
         <v>134</v>
       </c>
       <c r="D63" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E63" t="s">
-        <v>218</v>
+        <v>207</v>
       </c>
       <c r="F63" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G63" t="s">
         <v>134</v>
       </c>
       <c r="H63" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I63" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="64" spans="1:9">
@@ -2884,25 +2849,25 @@
         <v>118</v>
       </c>
       <c r="C64" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D64" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E64" t="s">
-        <v>219</v>
+        <v>208</v>
       </c>
       <c r="F64" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G64" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="H64" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I64" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="65" spans="1:9">
@@ -2913,25 +2878,25 @@
         <v>119</v>
       </c>
       <c r="C65" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="D65" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E65" t="s">
-        <v>220</v>
+        <v>209</v>
       </c>
       <c r="F65" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G65" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="H65" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I65" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="66" spans="1:9">
@@ -2942,22 +2907,22 @@
         <v>119</v>
       </c>
       <c r="C66" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D66" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="F66" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G66" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="H66" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I66" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="67" spans="1:9">
@@ -2968,22 +2933,22 @@
         <v>120</v>
       </c>
       <c r="C67" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="D67" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="F67" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G67" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="H67" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I67" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="68" spans="1:9">
@@ -2997,22 +2962,22 @@
         <v>134</v>
       </c>
       <c r="D68" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E68" t="s">
-        <v>221</v>
+        <v>210</v>
       </c>
       <c r="F68" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G68" t="s">
         <v>134</v>
       </c>
       <c r="H68" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I68" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="69" spans="1:9">
@@ -3023,25 +2988,25 @@
         <v>109</v>
       </c>
       <c r="C69" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="D69" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E69" t="s">
-        <v>222</v>
+        <v>211</v>
       </c>
       <c r="F69" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G69" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H69" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I69" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="70" spans="1:9">
@@ -3052,25 +3017,25 @@
         <v>122</v>
       </c>
       <c r="C70" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="D70" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E70" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="F70" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G70" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="H70" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I70" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="71" spans="1:9">
@@ -3081,25 +3046,25 @@
         <v>123</v>
       </c>
       <c r="C71" t="s">
+        <v>137</v>
+      </c>
+      <c r="D71" t="s">
         <v>148</v>
       </c>
-      <c r="D71" t="s">
-        <v>159</v>
-      </c>
       <c r="E71" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="F71" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G71" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="H71" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I71" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="72" spans="1:9">
@@ -3113,22 +3078,22 @@
         <v>134</v>
       </c>
       <c r="D72" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="E72" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="F72" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G72" t="s">
         <v>134</v>
       </c>
       <c r="H72" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I72" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="73" spans="1:9">
@@ -3139,25 +3104,25 @@
         <v>125</v>
       </c>
       <c r="C73" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D73" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E73" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="F73" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G73" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="H73" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I73" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="74" spans="1:9">
@@ -3168,25 +3133,25 @@
         <v>126</v>
       </c>
       <c r="C74" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="D74" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
       <c r="E74" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="F74" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G74" t="s">
-        <v>152</v>
+        <v>133</v>
       </c>
       <c r="H74" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I74" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="75" spans="1:9">
@@ -3197,25 +3162,25 @@
         <v>126</v>
       </c>
       <c r="C75" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="D75" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E75" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="F75" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G75" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="H75" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I75" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="76" spans="1:9">
@@ -3226,25 +3191,25 @@
         <v>127</v>
       </c>
       <c r="C76" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="D76" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E76" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="F76" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G76" t="s">
-        <v>154</v>
+        <v>139</v>
       </c>
       <c r="H76" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I76" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="77" spans="1:9">
@@ -3258,16 +3223,19 @@
         <v>139</v>
       </c>
       <c r="E77" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="F77" t="s">
-        <v>239</v>
+        <v>228</v>
+      </c>
+      <c r="G77" t="s">
+        <v>139</v>
       </c>
       <c r="H77" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
       <c r="I77" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="78" spans="1:9">
@@ -3281,22 +3249,22 @@
         <v>131</v>
       </c>
       <c r="D78" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="E78" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="F78" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G78" t="s">
         <v>131</v>
       </c>
       <c r="H78" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I78" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="79" spans="1:9">
@@ -3310,22 +3278,22 @@
         <v>134</v>
       </c>
       <c r="D79" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E79" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="F79" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G79" t="s">
         <v>134</v>
       </c>
       <c r="H79" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I79" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="80" spans="1:9">
@@ -3339,22 +3307,22 @@
         <v>138</v>
       </c>
       <c r="D80" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E80" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="F80" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G80" t="s">
         <v>138</v>
       </c>
       <c r="H80" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I80" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="81" spans="1:9">
@@ -3368,22 +3336,22 @@
         <v>138</v>
       </c>
       <c r="D81" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E81" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="F81" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G81" t="s">
         <v>138</v>
       </c>
       <c r="H81" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I81" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="82" spans="1:9">
@@ -3397,22 +3365,22 @@
         <v>138</v>
       </c>
       <c r="D82" t="s">
-        <v>164</v>
+        <v>153</v>
       </c>
       <c r="E82" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="F82" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G82" t="s">
         <v>138</v>
       </c>
       <c r="H82" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I82" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="83" spans="1:9">
@@ -3426,22 +3394,22 @@
         <v>138</v>
       </c>
       <c r="D83" t="s">
-        <v>159</v>
+        <v>148</v>
       </c>
       <c r="E83" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="F83" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G83" t="s">
         <v>138</v>
       </c>
       <c r="H83" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I83" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="84" spans="1:9">
@@ -3452,25 +3420,25 @@
         <v>128</v>
       </c>
       <c r="C84" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="D84" t="s">
-        <v>165</v>
+        <v>154</v>
       </c>
       <c r="E84" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="F84" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G84" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="H84" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I84" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="85" spans="1:9">
@@ -3484,22 +3452,22 @@
         <v>131</v>
       </c>
       <c r="D85" t="s">
-        <v>156</v>
+        <v>145</v>
       </c>
       <c r="E85" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="F85" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="G85" t="s">
         <v>131</v>
       </c>
       <c r="H85" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
       <c r="I85" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>